<commit_message>
updated data(3 Feb 2026) + dashboard update
</commit_message>
<xml_diff>
--- a/data/listings.xlsx
+++ b/data/listings.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:23</t>
+          <t>03-02-2026 12:14:45</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:23</t>
+          <t>03-02-2026 12:14:45</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:46</t>
+          <t>03-02-2026 12:15:11</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:48</t>
+          <t>03-02-2026 12:15:13</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -914,7 +914,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:43:43</t>
+          <t>03-02-2026 12:15:06</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:01</t>
+          <t>03-02-2026 12:15:25</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1322,7 +1322,7 @@
           <t>R 49,950</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="inlineStr">
         <is>
           <t>29,849km</t>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:03</t>
+          <t>03-02-2026 12:15:28</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:14</t>
+          <t>03-02-2026 12:15:39</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:34</t>
+          <t>03-02-2026 12:16:08</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:31</t>
+          <t>03-02-2026 12:16:03</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:46</t>
+          <t>03-02-2026 12:16:18</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -1631,7 +1631,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:46</t>
+          <t>03-02-2026 12:16:18</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:44:46</t>
+          <t>03-02-2026 12:16:18</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -1713,28 +1713,28 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Yamaha raptor 700</t>
+          <t>2016 xsr 700 Yamaha</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>R 76,900</t>
+          <t>R 110,000</t>
         </is>
       </c>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>6km</t>
+          <t>29,560km</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Thabazimbi</t>
+          <t>Mosselbaai</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>https://www.gumtree.co.za/a-motorcycles-scooters/thabazimbi/yamaha-raptor-700/10013461863741013316472309</t>
+          <t>https://www.gumtree.co.za/a-motorcycles-scooters/mosselbaai/2016-xsr-700-yamaha/10013466040191011073853909</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:06</t>
+          <t>03-02-2026 12:16:38</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>gumtree_10013461863741013316472309</t>
+          <t>gumtree_10013466040191011073853909</t>
         </is>
       </c>
     </row>
@@ -1766,28 +1766,28 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2016 xsr 700 Yamaha</t>
+          <t>Yamaha raptor 700</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>R 110,000</t>
+          <t>R 76,900</t>
         </is>
       </c>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>29,560km</t>
+          <t>6km</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Mosselbaai</t>
+          <t>Thabazimbi</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>https://www.gumtree.co.za/a-motorcycles-scooters/mosselbaai/2016-xsr-700-yamaha/10013466040191011073853909</t>
+          <t>https://www.gumtree.co.za/a-motorcycles-scooters/thabazimbi/yamaha-raptor-700/10013461863741013316472309</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -1797,12 +1797,12 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:03</t>
+          <t>03-02-2026 12:16:40</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>gumtree_10013466040191011073853909</t>
+          <t>gumtree_10013461863741013316472309</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:20</t>
+          <t>03-02-2026 12:16:52</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:20</t>
+          <t>03-02-2026 12:16:52</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:27</t>
+          <t>03-02-2026 12:16:59</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:26</t>
+          <t>03-02-2026 12:16:57</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:43</t>
+          <t>03-02-2026 12:17:17</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -2105,28 +2105,28 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>2018 BMW G310 GS</t>
+          <t>BMW 310</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>R 55,000</t>
+          <t>R 69,500</t>
         </is>
       </c>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>7,353km</t>
+          <t>17,000km</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Pietermaritzburg</t>
+          <t>Montague Gardens</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>https://www.gumtree.co.za/a-motorcycles-scooters/pietermaritzburg/2018-bmw-g310-gs/10013465574691012895313109</t>
+          <t>https://www.gumtree.co.za/a-motorcycles-scooters/montague-gardens/bmw-310/10013251672391010002889209</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2136,12 +2136,12 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:44</t>
+          <t>03-02-2026 12:17:17</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>gumtree_10013465574691012895313109</t>
+          <t>gumtree_10013251672391010002889209</t>
         </is>
       </c>
     </row>
@@ -2158,28 +2158,28 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>BMW 310</t>
+          <t>2018 BMW G310 GS</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>R 69,500</t>
+          <t>R 55,000</t>
         </is>
       </c>
       <c r="E41" s="4" t="n"/>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>17,000km</t>
+          <t>7,353km</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Montague Gardens</t>
+          <t>Pietermaritzburg</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>https://www.gumtree.co.za/a-motorcycles-scooters/montague-gardens/bmw-310/10013251672391010002889209</t>
+          <t>https://www.gumtree.co.za/a-motorcycles-scooters/pietermaritzburg/2018-bmw-g310-gs/10013465574691012895313109</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:43</t>
+          <t>03-02-2026 12:17:19</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>gumtree_10013251672391010002889209</t>
+          <t>gumtree_10013465574691012895313109</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:40</t>
+          <t>03-02-2026 12:17:13</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:40</t>
+          <t>03-02-2026 12:17:13</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:40</t>
+          <t>03-02-2026 12:17:13</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:40</t>
+          <t>03-02-2026 12:17:13</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:40</t>
+          <t>03-02-2026 12:17:13</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:55</t>
+          <t>03-02-2026 12:17:30</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:56</t>
+          <t>03-02-2026 12:17:32</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
@@ -2620,7 +2620,7 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:45:57</t>
+          <t>03-02-2026 12:17:33</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:46:12</t>
+          <t>03-02-2026 12:17:48</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
@@ -2710,7 +2710,7 @@
           <t>R 49,950</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr"/>
+      <c r="E53" s="4" t="n"/>
       <c r="F53" s="4" t="inlineStr">
         <is>
           <t>29,849km</t>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:46:12</t>
+          <t>03-02-2026 12:17:48</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:46:08</t>
+          <t>03-02-2026 12:17:44</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
@@ -2839,7 +2839,7 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>02-02-2026 21:46:08</t>
+          <t>03-02-2026 12:17:44</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>02/02/2026 21:46:28</t>
+          <t>03/02/2026 12:18:05</t>
         </is>
       </c>
     </row>

</xml_diff>